<commit_message>
revised helm chartts, and added new diagrams
</commit_message>
<xml_diff>
--- a/backend/docs/devops/Amendia_Component_Inventory_DevOps.xlsx
+++ b/backend/docs/devops/Amendia_Component_Inventory_DevOps.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,11 +80,6 @@
       <color rgb="FF1A1A1A"/>
       <sz val="15"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FFC00000"/>
-      <sz val="10"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -116,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,9 +142,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -614,7 +606,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Dev = docker-compose (this workbook's tabs 2–3). Prod = the portable umbrella Helm chart at deploy/helm/amendia (ADR-022) — see the 'Production (Helm)' tab. NOTE: the chart is at v0.1.0 and does NOT yet template glea-service or ClickHouse.</t>
+          <t>Dev = docker-compose (this workbook's tabs 2–3). Prod = the portable umbrella Helm chart at deploy/helm/amendia (ADR-022) — see the 'Production (Helm)' tab. Chart 0.2.0 (ADR-022 revision, 2026-08-19) now templates glea-service + ClickHouse with PVC-backed persistence.</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1303,7 @@
     <row r="48" ht="28" customHeight="1">
       <c r="A48" s="12" t="inlineStr">
         <is>
-          <t>•  ⚠  Helm chart gap: deploy/helm/amendia templates 8 services + capability-worker but NOT glea-service, and deploys no ClickHouse. ADR-058/063/064 audit has no prod packaging yet. Its otel collector also uses the non-contrib image (no ClickHouse exporter).</t>
+          <t>•  ⚠  glea-service has NO authentication layer (no amendia_auth dependency, no principal in any Depends). Its audit / decision-trail / lineage / cohort read APIs are open to anything that can reach the service. Restrict at the network layer; raised to the ADR-065 / PII workstream.</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1350,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Host ports corrected to the 18xxx map. stub-exception-generator renamed stub-trigger-generator (ADR-059) with its queue (ingestor.trigger_raised.v1) and dispatch queue (agent-runtime.trigger_dispatched.v1). notification-service corrected: it is SSE-only — it does NOT route Slack/Teams/email (no such sender exists in the platform; backlog CB-7). Env var names given their service prefixes. Added the 3 ACH MCP servers (8075–8077), pega-stub (9095), glea-service's cohort_events + cohort_sla_events tables (ADR-063/064) and the agent-runtime cohort/SLA Mongo collections. New 'Production (Helm)' tab. Added the real-Bedrock-egress and Helm-coverage warnings.</t>
+          <t>Host ports corrected to the 18xxx map. stub-exception-generator renamed stub-trigger-generator (ADR-059) with its queue (ingestor.trigger_raised.v1) and dispatch queue (agent-runtime.trigger_dispatched.v1). notification-service corrected: it is SSE-only — it does NOT route Slack/Teams/email (no such sender exists in the platform; backlog CB-7). Env var names given their service prefixes. Added the 3 ACH MCP servers (8075–8077), pega-stub (9095), glea-service's cohort_events + cohort_sla_events tables (ADR-063/064) and the agent-runtime cohort/SLA Mongo collections. New 'Production (Helm)' tab. Added the real-Bedrock-egress and Helm-coverage warnings.  Later on 2026-08-19: glea-service Auth corrected — v1 said "Keycloak JWT (read APIs)", verified false, it has no auth layer. Production (Helm) tab updated to chart 0.2.0 after the ADR-022 catch-up.</t>
         </is>
       </c>
     </row>
@@ -1973,17 +1965,17 @@
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>Keycloak JWT (read APIs)</t>
+          <t>⚠ NONE — no auth layer at all</t>
         </is>
       </c>
       <c r="K12" s="10" t="inlineStr">
         <is>
-          <t>GLEA_RABBITMQ_URL; GLEA_CLICKHOUSE_HOST=clickhouse; GLEA_CLICKHOUSE_PORT=8123; GLEA_CLICKHOUSE_DB=glea; SEALING_INTERVAL_SECONDS=30; OTLP endpoint</t>
+          <t>GLEA_RABBITMQ_URL; GLEA_CLICKHOUSE_HOST=clickhouse; GLEA_CLICKHOUSE_PORT=8123; GLEA_CLICKHOUSE_DB=glea; GLEA_AUDIT_TTL_DAYS=2555 (~7 yr); SEALING_INTERVAL_SECONDS=30; OTLP endpoint</t>
         </is>
       </c>
       <c r="L12" s="10" t="inlineStr">
         <is>
-          <t>ADR-058/063/064. Durable NAMED RabbitMQ queue (competing consumers) — must not lose messages; this is the queue the missing RabbitMQ volume puts at risk. Background hash-chain sealer (prev_hash/seal columns are declared but NOT yet written — the chain is scaffolded, inert). Bounded ClickHouse connection pool. ⚠ NOT templated in the Helm chart — no prod packaging yet.</t>
+          <t>⚠ CORRECTION vs v1: glea-service has NO authentication. config.py declares no *_AUTH_* or *_INTERNAL_TOKEN, amendia_auth is not in its pyproject.toml, nothing under app/ imports it, and every Depends() injects a reader/consumer rather than a principal — so the audit trail, decision trails, lineage and cohort/SLA read-models are readable by anything that can reach :8090. Restrict at the network layer until decided (raised to the ADR-065 / PII workstream). ADR-058/063/064. Durable NAMED RabbitMQ queue (competing consumers) — must not lose messages; this is the queue the missing RabbitMQ volume puts at risk. Background hash-chain sealer (prev_hash/seal columns are declared but NOT yet written — the chain is scaffolded, inert). Bounded ClickHouse connection pool. ⚠ NOT templated in the Helm chart — no prod packaging yet.</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2740,7 @@
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>STATEFUL — back up clickhouse_data. Native port remapped 9001(host)→9000(container). TTLs: audit multi-year (~7 yr), traces short. Sole writer of the audit tables = glea-service. ⚠ Not deployed by the Helm chart — prod ClickHouse must be provisioned separately.</t>
+          <t>STATEFUL — back up clickhouse_data. Native port remapped 9001(host)→9000(container). TTLs: audit multi-year (~7 yr), traces short. Sole writer of the audit tables = glea-service. Deployed by Helm as of chart 0.2.0 (datastores.clickhouse, 8123+9000, 50Gi PVC) — set deploy:false to point at a managed ClickHouse.</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2797,7 @@
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>Stateless — scale/replace freely. REQUIRES the -contrib image for the ClickHouse exporter. Command: --config=/etc/otel/collector-config.yaml. Services point AGENTRT_OTLP_ENDPOINT / *_OTLP_ENDPOINT here (:4318). ⚠ Pipeline is `processors: [batch]` only — no attributes/redaction/filter/transform processor, so nothing scrubs sensitive values out of traces. ⚠ The Helm chart pins the NON-contrib image, which cannot export to ClickHouse.</t>
+          <t>Stateless — scale/replace freely. REQUIRES the -contrib image for the ClickHouse exporter. Command: --config=/etc/otel/collector-config.yaml. Services point AGENTRT_OTLP_ENDPOINT / *_OTLP_ENDPOINT here (:4318). ⚠ Pipeline is `processors: [batch]` only — no attributes/redaction/filter/transform processor, so nothing scrubs sensitive values out of traces. The Helm chart now pins the same -contrib image and exports traces + logs to ClickHouse (chart 0.2.0).</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2897,7 +2889,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The portable umbrella chart at deploy/helm/amendia (chart 0.1.0, appVersion 0.1.0) + Vault config at deploy/vault. Generic base + thin per-provider values overlays. Read-verified 2026-08-19. NEW in v2 of this workbook.</t>
+          <t>The portable umbrella chart at deploy/helm/amendia (chart 0.2.0, appVersion 0.1.0) + Vault config at deploy/vault. Generic base + thin per-provider values overlays. Read-verified 2026-08-19. NEW in v2 of this workbook.</t>
         </is>
       </c>
     </row>
@@ -2992,732 +2984,752 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>As of chart 0.2.0, any datastore with deploy:true and a storage value renders a PVC (RWO; storageClassName omitted when global.storageClass="" so the cluster default applies): mongodb 10Gi /data/db, rabbitmq 8Gi /var/lib/rabbitmq, clickhouse 50Gi /var/lib/clickhouse. ⚠ These Deployments still use the default RollingUpdate strategy — set strategy: Recreate before the first helm upgrade, or an RWO volume will deadlock the rollout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Templated services (values.services.*)</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Port · env prefix · health</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Egress allowlist</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Vault secretEnv</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>stub-trigger-generator</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>8081 · STUBTRIG · /health</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>mongodb, rabbitmq, identity</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>STUBTRIG_AUTH_INTERNAL_TOKEN, RABBIT_USER, RABBIT_PASSWORD</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>MONGO_COLLECTION=trigger_messages. Dev/test stub — normally replaced by the real source connector.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>ingestor</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>8082 · INGESTOR · /health</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>mongodb, rabbitmq, process-registry, stub-trigger-generator, identity</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>INGESTOR_AUTH_INTERNAL_TOKEN, RABBIT_USER, RABBIT_PASSWORD</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>Queue ingestor.trigger_raised.v1; reply ingestor.dispatch_replies.v1.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>agent-runtime</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>8083 · AGENTRT · /health</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>mongodb, rabbitmq, process-registry, config-forge, identity, otel</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>AGENTRT_AUTH_INTERNAL_TOKEN, RABBIT_USER, RABBIT_PASSWORD, AWS_ACCESS_KEY_ID, AWS_SECRET_ACCESS_KEY, NVIDIA_NIM_API_KEY, OPENSHELL_INFERENCE_TOKEN</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Prod locks down the dev escape hatches: ENABLE_SEED_API=false, ENABLE_DEBUG_API=false, ENABLE_DEV_CORS=false. SIMULATION_MODE=false.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>process-registry</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>8084 · REGISTRY · /health</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>mongodb, identity</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>REGISTRY_AUTH_INTERNAL_TOKEN</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>SEED_ON_STARTUP=true.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>identity</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>8086 · IDENTITY · /health</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>mongodb, keycloak</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>IDENTITY_INTERNAL_TOKEN</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>SEED_ON_STARTUP=true; JIT_DEFAULT_STATUS=active.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>notification-service</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>8088 · NOTIFICATION · /health</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>rabbitmq, identity</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>NOTIFICATION_AUTH_INTERNAL_TOKEN, RABBIT_USER, RABBIT_PASSWORD</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>SSE fan-out only — no email/chat sender exists.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>config-forge</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>8040 · (unprefixed) · /healthz</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>mongodb</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>— (none)</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>common:false → unprefixed env (MONGO_URI, MONGO_DB=ConfigForge, SERVICE_NAME, PORT, ENV=prod). Health is /healthz.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>webui</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>8085 · (static) · /</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
         <is>
           <t>stub-trigger-generator, ingestor, agent-runtime, process-registry, notification-service</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>— (none)</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>nginx SPA, no app env (static:true).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>capability-worker</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>no Service/port · AGENTRT · n/a (broker consumer)</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>rabbitmq, config-forge, inference, mcp, otel</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>RABBIT_USER, RABBIT_PASSWORD, AWS_ACCESS_KEY_ID, AWS_SECRET_ACCESS_KEY, NVIDIA_NIM_API_KEY, OPENSHELL_INFERENCE_TOKEN</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>Rendered only when executionMode=nemoclaw. replicas 2 = the ADR-020 warm pool. Same image as agent-runtime, command python -m worker.main.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>glea-service</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>⚠ NOT TEMPLATED</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>8090 · GLEA · /health</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>rabbitmq, clickhouse, otel</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>RABBIT_USER, RABBIT_PASSWORD</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Added in chart 0.2.0 (ADR-022 revision, 2026-08-19) as a pure values entry — no new template. No mongoDb, no identity egress, no internal token: glea has no auth layer. ClickHouse settings via extraEnv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Optional in-cluster datastores (datastores.*)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>mongodb</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>deploy: true</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>mongo:7</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>10Gi (global.storageClass)</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Override to a managed endpoint (Atlas / DocumentDB / CosmosDB) via mongo.uri.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>rabbitmq</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>deploy: true</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>rabbitmq:3-management</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>— (no PVC in chart)</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>user/password come from Vault; host is the in-cluster Service or BYO/managed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>keycloak</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>deploy: false</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>quay.io/keycloak/keycloak:26.0</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>⚠ GAP: the chart predates ADR-058 and does not render glea-service, nor any ClickHouse datastore. The audit system-of-record (audit_events, cohort_events, cohort_sla_events) has no production packaging today.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Optional in-cluster datastores (datastores.*)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Image</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>mongodb</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Usually external/managed in prod — this is the customer's own IAM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>clickhouse</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>deploy: true</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>mongo:7</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>10Gi (global.storageClass)</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Override to a managed endpoint (Atlas / DocumentDB / CosmosDB) via mongo.uri.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>rabbitmq</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>deploy: true</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>rabbitmq:3-management</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>— (no PVC in chart)</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>user/password come from Vault; host is the in-cluster Service or BYO/managed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>keycloak</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>deploy: false</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>quay.io/keycloak/keycloak:26.0</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Usually external/managed in prod — this is the customer's own IAM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="14" t="inlineStr">
-        <is>
-          <t>clickhouse</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>⚠ absent</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D31" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>Not in the chart at all. Must be provisioned separately for GLEA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>clickhouse/clickhouse-server:24.8</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>50Gi PVC → /var/lib/clickhouse</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Added in chart 0.2.0. Ports 8123 (HTTP, GLEA) + 9000 (native, collector). 50Gi is a sizing seam against the ~7-yr audit TTL, not a computed guarantee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Secrets — Vault (Kubernetes auth)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Why K8s auth</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Portable across GKE/EKS/AKS/on-prem: pods authenticate with their Kubernetes ServiceAccount, so secrets need no per-cloud workload-identity dependency. Realizes ADR-016's literal: → vault: migration. No plaintext secret in Git, values, or a bare K8s Secret.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Delivery method</t>
+          <t>Why K8s auth</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>⚠ Inconsistency to resolve: values.yaml sets vault.method="agent-injector", but deploy/vault/README.md states "CSI is the default". Pick one before handover. csi → Secrets Store CSI driver syncs each service's Vault path into a per-service Secret consumed via secretKeyRef (chart renders a SecretProviderClass per service). agent-injector → secrets rendered into /vault/secrets/ via pod annotations.</t>
+          <t>Portable across GKE/EKS/AKS/on-prem: pods authenticate with their Kubernetes ServiceAccount, so secrets need no per-cloud workload-identity dependency. Realizes ADR-016's literal: → vault: migration. No plaintext secret in Git, values, or a bare K8s Secret.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Role &amp; paths</t>
+          <t>Delivery method</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>One Vault role 'amendia' bound to all 9 Amendia ServiceAccounts in namespace 'amendia', ttl 1h. Policy grants read-only on secret/data/amendia/&lt;service&gt; per service, plus secret/data/amendia/nim for NGC_API_KEY.</t>
+          <t>vault.method="csi" (default as of chart 0.2.0 — previously agent-injector, which contradicted the docs and rendered zero SecretProviderClasses). csi → Secrets Store CSI driver syncs each service's Vault path into a per-service Secret consumed via secretKeyRef, one SecretProviderClass per service. agent-injector remains the documented alternative: secrets rendered into /vault/secrets/ via pod annotations.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Least-privilege note</t>
+          <t>Role &amp; paths</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>The shipped policy.hcl is a single shared policy — any bound service could read another's path. deploy/vault/README.md flags this: split into one policy per ServiceAccount to tighten.</t>
+          <t>One Vault role 'amendia' bound to all 9 Amendia ServiceAccounts in namespace 'amendia', ttl 1h. Policy grants read-only on secret/data/amendia/&lt;service&gt; per service, plus secret/data/amendia/nim for NGC_API_KEY.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
+          <t>Least-privilege note</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>The shipped policy.hcl is a single shared policy — any bound service could read another's path. deploy/vault/README.md flags this: split into one policy per ServiceAccount to tighten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
           <t>Address / base path</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>vault.address=https://vault.amendia.example (per-deployment); secretBasePath=secret/data/amendia (KV-v2).</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>Network policy &amp; egress</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>Posture</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>networkPolicy.enabled=true, defaultDenyEgress=true, allowDNS=true (kube-dns required for Service resolution). Each service's allowlist comes from its values 'egress' list (see the table above).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Per-provider caveat</t>
+          <t>Posture</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>CNI differences (Calico / Cilium / GKE-native) may need extra ipBlocks — flagged as a '# per-provider' seam.</t>
+          <t>networkPolicy.enabled=true, defaultDenyEgress=true, allowDNS=true (kube-dns required for Service resolution). Each service's allowlist comes from its values 'egress' list (see the table above).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
+          <t>Per-provider caveat</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>CNI differences (Calico / Cilium / GKE-native) may need extra ipBlocks — flagged as a '# per-provider' seam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
           <t>Gap</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>⚠ No egress rule exists for glea-service or ClickHouse, since neither is templated. Adding GLEA to the chart means adding its allowlist and the ClickHouse endpoint too.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>Inference serving (one toggle — ADR-018/022 Part C)</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="6" t="inlineStr">
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>inference.mode</t>
         </is>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>Active ConfigForge LLM ref</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Where it runs</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>nim-selfhosted (default)</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>prod.llm.nemoclaw.nemotron-ultra</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>In-cluster NIM workload (amendia-nim:8000)</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>nvcr.io/nim/nvidia/nemotron-3-ultra:latest, limits nvidia.com/gpu: 1, GPU nodeSelector/tolerations per provider. Marked # [confirm] against NVIDIA's official NIM Helm packaging.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="9" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
         <is>
           <t>nvidia-hosted</t>
         </is>
       </c>
-      <c r="B48" s="10" t="inlineStr">
+      <c r="B49" s="10" t="inlineStr">
         <is>
           <t>prod.llm.nemoclaw.nim</t>
         </is>
       </c>
-      <c r="C48" s="10" t="inlineStr">
+      <c r="C49" s="10" t="inlineStr">
         <is>
           <t>https://integrate.api.nvidia.com/v1</t>
         </is>
       </c>
-      <c r="D48" s="10" t="inlineStr">
+      <c r="D49" s="10" t="inlineStr">
         <is>
           <t>Managed NVIDIA endpoint — outbound egress from the cluster.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>bedrock-only</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>prod.llm.bedrock.explicit-creds</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>AWS Bedrock</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>No cluster GPU. This is the mode the dev compose stack effectively runs today (us-east-1).</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>Seed job</t>
         </is>
       </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>inference.seedJob.enabled=true renders configforge-seed-job.yaml, which PUTs the active ref's base_url into ConfigForge so the worker resolves it (ADR-018).</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>Known gaps to close before a real production handover</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="28" customHeight="1">
-      <c r="A53" s="12" t="inlineStr">
-        <is>
-          <t>1.  glea-service and ClickHouse are not in the chart — the ADR-058/063/064 audit system-of-record has no prod packaging, no Service, no NetworkPolicy and no storage plan.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="28" customHeight="1">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>2.  otel.collectorImage pins otel/opentelemetry-collector:0.109.0 (NON-contrib). The ClickHouse exporter used in compose needs the -contrib image; as configured, prod traces cannot land in ClickHouse.</t>
+          <t>1.  ⚠ OPEN: the new PVC-backed datastore Deployments keep the default RollingUpdate strategy. With replicas:1, maxSurge=1/maxUnavailable=0 schedules the replacement pod before the old one releases the RWO volume — the rollout deadlocks on a single-attach CSI driver. Set strategy: {type: Recreate}, or move ClickHouse/Mongo to StatefulSets. Bites on the first helm upgrade, not a fresh install.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="28" customHeight="1">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>3.  vault.method disagrees between values.yaml (agent-injector) and deploy/vault/README.md (CSI is the default).</t>
+          <t>2.  glea-service has no authentication of its own (see the Custom Services tab). Nothing in this chart restricts who may call the audit read APIs in-cluster — NetworkPolicies here govern egress, not ingress.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t>4.  openshell.sandbox.enabled=false and carries an explicit '# [confirm] + STOP' — NemoClaw's K8s sandbox mechanism is unconfirmed. The baseline (hardened worker Deployment + NetworkPolicy) is the supported posture.</t>
+          <t>3.  ClickHouse is a single-replica Deployment with the passwordless 'default' user and inherits defaults.resources (cpu 1 / mem 512Mi). All three want revisiting before a real audit workload; GLEA_CLICKHOUSE_PASSWORD is not wired to Vault.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t>5.  The NIM image/args/licensing line is marked # [confirm] against NVIDIA's Helm packaging.</t>
+          <t>4.  With datastores.clickhouse.deploy=false, glea's GLEA_CLICKHOUSE_HOST and otel.clickhouse.endpoint must be overridden separately — a single clickhouse.host seam (as mongo.uri / rabbit.host do) would repoint both.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="12" t="inlineStr">
         <is>
-          <t>6.  Vault policy.hcl is one shared policy across all ServiceAccounts — tighten to per-SA policies for true least privilege.</t>
+          <t>5.  datastores.keycloak still has no storage value — ephemeral wherever it is deployed in-cluster (on-prem overlay).</t>
         </is>
       </c>
     </row>
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>7.  Chart is v0.1.0 and has not been revised since ADR-022; it predates ADR-058 through ADR-064. Treat it as a scaffold, not a shipped artifact.</t>
+          <t>6.  openshell.sandbox.enabled=false carries an explicit '# [confirm] + STOP' — NemoClaw's K8s sandbox mechanism is unconfirmed. The baseline (hardened worker Deployment + NetworkPolicy) is the supported posture. The NIM image/args/licensing line is likewise # [confirm].</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1">
+      <c r="A60" s="12" t="inlineStr">
+        <is>
+          <t>7.  Vault policy.hcl is one shared policy across all ServiceAccounts — tighten to per-SA policies for true least privilege.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="28" customHeight="1">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>8.  Everything on this tab is a helm template / helm lint result. No runtime behaviour has been verified — no cluster, no image pull, no ClickHouse round-trip.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A53:E53"/>
+  <mergeCells count="8">
     <mergeCell ref="A55:E55"/>
     <mergeCell ref="A59:E59"/>
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A61:E61"/>
     <mergeCell ref="A58:E58"/>
     <mergeCell ref="A56:E56"/>
   </mergeCells>

</xml_diff>